<commit_message>
Try-improve-AltGr-key-operation - revert previous commit - add reactions on event->state
</commit_message>
<xml_diff>
--- a/src/index spreadsheet/GTK key codes.xlsx
+++ b/src/index spreadsheet/GTK key codes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacomostert/wp43s/src/index spreadsheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F1B2C8-6BE6-2E46-B954-FE94A0CE4B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E8ED3B-C15D-DC4C-A7A1-AB95631BAD3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4660" yWindow="3400" windowWidth="28040" windowHeight="17440" xr2:uid="{E19FABB6-FEBD-1F48-A261-18932C58251D}"/>
   </bookViews>
@@ -15828,6 +15828,21 @@
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
+      <c r="E4">
+        <v>65505</v>
+      </c>
+      <c r="F4" t="str">
+        <f>DEC2HEX(E4)</f>
+        <v>FFE1</v>
+      </c>
+      <c r="G4">
+        <f>MATCH(E4,D:D,0)</f>
+        <v>1358</v>
+      </c>
+      <c r="H4" t="str" cm="1">
+        <f t="array" ref="H4">INDEX(B:B,G4)</f>
+        <v>GDK_KEY_Shift_L</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -15845,19 +15860,19 @@
         <v>36</v>
       </c>
       <c r="E5">
-        <v>65505</v>
+        <v>65506</v>
       </c>
       <c r="F5" t="str">
         <f>DEC2HEX(E5)</f>
-        <v>FFE1</v>
+        <v>FFE2</v>
       </c>
       <c r="G5">
         <f>MATCH(E5,D:D,0)</f>
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="H5" t="str" cm="1">
         <f t="array" ref="H5">INDEX(B:B,G5)</f>
-        <v>GDK_KEY_Shift_L</v>
+        <v>GDK_KEY_Shift_R</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -15998,6 +16013,21 @@
       <c r="D10">
         <f t="shared" si="1"/>
         <v>40</v>
+      </c>
+      <c r="E10">
+        <v>65513</v>
+      </c>
+      <c r="F10" t="str">
+        <f>DEC2HEX(E10)</f>
+        <v>FFE9</v>
+      </c>
+      <c r="G10">
+        <f>MATCH(E10,D:D,0)</f>
+        <v>1366</v>
+      </c>
+      <c r="H10" t="str" cm="1">
+        <f t="array" ref="H10">INDEX(B:B,G10)</f>
+        <v>GDK_KEY_Alt_L</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>